<commit_message>
Landed-cost building blocks: new slide (UA/EN V12) and sheet in SIAS model
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_SIAS_EN.xlsx
+++ b/RAMEN_FINMODEL_SIAS_EN.xlsx
@@ -6,8 +6,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 pallets" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="33 pallets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Landed cost blocks" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 pallets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="33 pallets" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,7 +17,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="20">
+  <numFmts count="21">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00&quot; ₴&quot;_-;\-* #,##0.00&quot; ₴&quot;_-;_-* \-??&quot; ₴&quot;_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00\ [$₴-422]_-;\-* #,##0.00\ [$₴-422]_-;_-* \-??\ [$₴-422]_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="0.0000&quot; €&quot;"/>
@@ -37,8 +38,9 @@
     <numFmt numFmtId="181" formatCode="_(* #,##0_);_(* \(#,##0\);_(* \-_);_(@_)"/>
     <numFmt numFmtId="182" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
     <numFmt numFmtId="183" formatCode="_(\$* #,##0_);_(\$* \(#,##0\);_(\$* \-_);_(@_)"/>
+    <numFmt numFmtId="184" formatCode="0.00;-0.00;&quot;OK&quot;"/>
   </numFmts>
-  <fonts count="41">
+  <fonts count="42">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -270,6 +272,11 @@
       <name val="Arial"/>
       <color rgb="FF0000FF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="30">
@@ -776,7 +783,7 @@
     <xf numFmtId="0" fontId="11" fillId="19" borderId="10"/>
     <xf numFmtId="9" fontId="1" fillId="19" borderId="10"/>
   </cellStyleXfs>
-  <cellXfs count="174">
+  <cellXfs count="182">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1252,6 +1259,26 @@
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="41" fillId="28" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="24" fillId="27" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="19" fillId="25" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="184" fontId="30" fillId="25" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="37" fillId="29" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="24" fillId="29" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="170" fontId="33" fillId="24" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1543,6 +1570,354 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" style="71" min="1" max="1"/>
+    <col width="17" customWidth="1" style="71" min="2" max="2"/>
+    <col width="17" customWidth="1" style="71" min="3" max="3"/>
+    <col width="17" customWidth="1" style="71" min="4" max="4"/>
+    <col width="17" customWidth="1" style="71" min="5" max="5"/>
+    <col width="17" customWidth="1" style="71" min="6" max="6"/>
+    <col width="17" customWidth="1" style="71" min="7" max="7"/>
+    <col width="17" customWidth="1" style="71" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" s="71">
+      <c r="A1" s="172" t="inlineStr">
+        <is>
+          <t>What the landed cost in Ukraine is made of · ₴ per pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1" s="71">
+      <c r="A2" s="154" t="inlineStr">
+        <is>
+          <t>SIAS purchase + delivery + import VAT + financing = landed cost. Delivery = freight, broker, terminal and certification of the batch, per pack. Customs duty 0 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="173" t="inlineStr">
+        <is>
+          <t>33 PALLETS · FULL TRUCK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1" s="71">
+      <c r="A5" s="161" t="inlineStr"/>
+      <c r="B5" s="161" t="inlineStr">
+        <is>
+          <t>SIAS purchase
+pack price × rate</t>
+        </is>
+      </c>
+      <c r="C5" s="161" t="inlineStr">
+        <is>
+          <t>Delivery
+freight, broker, terminal</t>
+        </is>
+      </c>
+      <c r="D5" s="161" t="inlineStr">
+        <is>
+          <t>Import VAT
+20 % on goods and freight</t>
+        </is>
+      </c>
+      <c r="E5" s="161" t="inlineStr">
+        <is>
+          <t>Financing
+2.5 % of the sum</t>
+        </is>
+      </c>
+      <c r="F5" s="161" t="inlineStr">
+        <is>
+          <t>Landed cost, ₴ (sum of blocks)</t>
+        </is>
+      </c>
+      <c r="G5" s="161" t="inlineStr">
+        <is>
+          <t>Landed cost, €</t>
+        </is>
+      </c>
+      <c r="H5" s="161" t="inlineStr">
+        <is>
+          <t>Check vs model sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1" s="71">
+      <c r="A6" s="163" t="inlineStr">
+        <is>
+          <t>BEFORE · 4 SKUs
+(Vegetable, Spicy, Beef, Chicken)</t>
+        </is>
+      </c>
+      <c r="B6" s="174" t="n">
+        <v>33.28</v>
+      </c>
+      <c r="C6" s="174" t="n">
+        <v>3.668446389496718</v>
+      </c>
+      <c r="D6" s="174" t="n">
+        <v>7.127527352297594</v>
+      </c>
+      <c r="E6" s="174" t="n">
+        <v>1.101899343544858</v>
+      </c>
+      <c r="F6" s="175">
+        <f>SUM(B6:E6)</f>
+        <v>45.17787308533917</v>
+      </c>
+      <c r="G6" s="176">
+        <f>F6/'33 pallets'!F14</f>
+        <v>0.8823803336980307</v>
+      </c>
+      <c r="H6" s="177">
+        <f>ROUND(F6-'33 pallets'!C4,4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1" s="71">
+      <c r="A7" s="163" t="inlineStr">
+        <is>
+          <t>BEFORE · 2 SKUs
+(Gouda, Carbonara)</t>
+        </is>
+      </c>
+      <c r="B7" s="174" t="n">
+        <v>38.40000000000001</v>
+      </c>
+      <c r="C7" s="174" t="n">
+        <v>4.232822757111598</v>
+      </c>
+      <c r="D7" s="174" t="n">
+        <v>8.22407002188184</v>
+      </c>
+      <c r="E7" s="174" t="n">
+        <v>1.271422319474836</v>
+      </c>
+      <c r="F7" s="175">
+        <f>SUM(B7:E7)</f>
+        <v>52.12831509846829</v>
+      </c>
+      <c r="G7" s="176">
+        <f>F7/'33 pallets'!F14</f>
+        <v>1.0181311542669587</v>
+      </c>
+      <c r="H7" s="177">
+        <f>ROUND(F7-'33 pallets'!C6,4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1" s="71">
+      <c r="A8" s="170" t="inlineStr">
+        <is>
+          <t>AFTER · SIAS request
+(all 6 SKUs)</t>
+        </is>
+      </c>
+      <c r="B8" s="178">
+        <f>'33 pallets'!B19*'33 pallets'!F14</f>
+        <v>27.648000000000003</v>
+      </c>
+      <c r="C8" s="178">
+        <f>('33 pallets'!E16+'33 pallets'!F16+'33 pallets'!G16)/('33 pallets'!C18*'33 pallets'!D18)*'33 pallets'!F14</f>
+        <v>3.907878787878788</v>
+      </c>
+      <c r="D8" s="178">
+        <f>('33 pallets'!B19+'33 pallets'!E16*'33 pallets'!B18/('33 pallets'!C18*'33 pallets'!D18))*(1+'33 pallets'!D16)*'33 pallets'!B16*'33 pallets'!F14</f>
+        <v>6.031903030303031</v>
+      </c>
+      <c r="E8" s="178">
+        <f>(B8+C8+D8+('33 pallets'!B19+'33 pallets'!E16*'33 pallets'!B18/('33 pallets'!C18*'33 pallets'!D18))*'33 pallets'!D16*'33 pallets'!F14)*'33 pallets'!C16</f>
+        <v>0.9396945454545457</v>
+      </c>
+      <c r="F8" s="179">
+        <f>SUM(B8:E8)</f>
+        <v>38.52747636363637</v>
+      </c>
+      <c r="G8" s="176">
+        <f>F8/'33 pallets'!F14</f>
+        <v>0.7524897727272728</v>
+      </c>
+      <c r="H8" s="177">
+        <f>ROUND(F8-'33 pallets'!C8,4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="173" t="inlineStr">
+        <is>
+          <t>6 PALLETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1" s="71">
+      <c r="A11" s="161" t="inlineStr"/>
+      <c r="B11" s="161" t="inlineStr">
+        <is>
+          <t>SIAS purchase
+pack price × rate</t>
+        </is>
+      </c>
+      <c r="C11" s="161" t="inlineStr">
+        <is>
+          <t>Delivery
+freight, broker, terminal</t>
+        </is>
+      </c>
+      <c r="D11" s="161" t="inlineStr">
+        <is>
+          <t>Import VAT
+20 % on goods and freight</t>
+        </is>
+      </c>
+      <c r="E11" s="161" t="inlineStr">
+        <is>
+          <t>Financing
+2.5 % of the sum</t>
+        </is>
+      </c>
+      <c r="F11" s="161" t="inlineStr">
+        <is>
+          <t>Landed cost, ₴ (sum of blocks)</t>
+        </is>
+      </c>
+      <c r="G11" s="161" t="inlineStr">
+        <is>
+          <t>Landed cost, €</t>
+        </is>
+      </c>
+      <c r="H11" s="161" t="inlineStr">
+        <is>
+          <t>Check vs model sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1" s="71">
+      <c r="A12" s="163" t="inlineStr">
+        <is>
+          <t>BEFORE · 4 SKUs
+(Vegetable, Spicy, Beef, Chicken)</t>
+        </is>
+      </c>
+      <c r="B12" s="174" t="n">
+        <v>33.28</v>
+      </c>
+      <c r="C12" s="174" t="n">
+        <v>14.86439024390244</v>
+      </c>
+      <c r="D12" s="174" t="n">
+        <v>8.502634146341462</v>
+      </c>
+      <c r="E12" s="174" t="n">
+        <v>1.416175609756098</v>
+      </c>
+      <c r="F12" s="175">
+        <f>SUM(B12:E12)</f>
+        <v>58.0632</v>
+      </c>
+      <c r="G12" s="176">
+        <f>F12/'6 pallets'!F14</f>
+        <v>1.134046875</v>
+      </c>
+      <c r="H12" s="177">
+        <f>ROUND(F12-'6 pallets'!C4,4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1" s="71">
+      <c r="A13" s="163" t="inlineStr">
+        <is>
+          <t>BEFORE · 2 SKUs
+(Gouda, Carbonara)</t>
+        </is>
+      </c>
+      <c r="B13" s="174" t="n">
+        <v>38.40000000000001</v>
+      </c>
+      <c r="C13" s="174" t="n">
+        <v>17.15121951219512</v>
+      </c>
+      <c r="D13" s="174" t="n">
+        <v>9.810731707317075</v>
+      </c>
+      <c r="E13" s="174" t="n">
+        <v>1.634048780487805</v>
+      </c>
+      <c r="F13" s="175">
+        <f>SUM(B13:E13)</f>
+        <v>66.99600000000001</v>
+      </c>
+      <c r="G13" s="176">
+        <f>F13/'6 pallets'!F14</f>
+        <v>1.308515625</v>
+      </c>
+      <c r="H13" s="177">
+        <f>ROUND(F13-'6 pallets'!C6,4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1" s="71">
+      <c r="A14" s="170" t="inlineStr">
+        <is>
+          <t>AFTER · SIAS request
+(all 6 SKUs)</t>
+        </is>
+      </c>
+      <c r="B14" s="178">
+        <f>'6 pallets'!B20*'6 pallets'!F14</f>
+        <v>16.384</v>
+      </c>
+      <c r="C14" s="178">
+        <f>('6 pallets'!E16+'6 pallets'!F16+'6 pallets'!G16)/('6 pallets'!C18*'6 pallets'!D18)*'6 pallets'!F14</f>
+        <v>15.626666666666669</v>
+      </c>
+      <c r="D14" s="178">
+        <f>('6 pallets'!B20+'6 pallets'!E16*'6 pallets'!B18/('6 pallets'!C18*'6 pallets'!D18))*(1+'6 pallets'!D16)*'6 pallets'!B16*'6 pallets'!F14</f>
+        <v>5.218133333333333</v>
+      </c>
+      <c r="E14" s="178">
+        <f>(B14+C14+D14+('6 pallets'!B20+'6 pallets'!E16*'6 pallets'!B18/('6 pallets'!C18*'6 pallets'!D18))*'6 pallets'!D16*'6 pallets'!F14)*'6 pallets'!C16</f>
+        <v>0.93072</v>
+      </c>
+      <c r="F14" s="179">
+        <f>SUM(B14:E14)</f>
+        <v>38.15952</v>
+      </c>
+      <c r="G14" s="176">
+        <f>F14/'6 pallets'!F14</f>
+        <v>0.745303125</v>
+      </c>
+      <c r="H14" s="177">
+        <f>ROUND(F14-'6 pallets'!C8,4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1" s="71">
+      <c r="A16" s="171" t="inlineStr">
+        <is>
+          <t>"Before": per our cost file (logistics allocated by value). "After": at the requested price, logistics spread evenly per pack. The smaller the batch, the higher the delivery cost per pack.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="FF223A5E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -1959,7 +2334,7 @@
       <c r="D14" s="145" t="n">
         <v>0.35</v>
       </c>
-      <c r="E14" s="172" t="n">
+      <c r="E14" s="180" t="n">
         <v>1.4</v>
       </c>
       <c r="F14" s="53" t="n">
@@ -2087,7 +2462,7 @@
           <t>Landed cost today, 4 SKUs (Vegetable, Spicy, Beef, Chicken), €/pack</t>
         </is>
       </c>
-      <c r="B24" s="173" t="n">
+      <c r="B24" s="181" t="n">
         <v>1.134046875</v>
       </c>
     </row>
@@ -2097,7 +2472,7 @@
           <t>Landed cost today, 2 SKUs (Gouda, Carbonara), €/pack</t>
         </is>
       </c>
-      <c r="B25" s="173" t="n">
+      <c r="B25" s="181" t="n">
         <v>1.308515625</v>
       </c>
     </row>
@@ -2118,7 +2493,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF223A5E"/>
@@ -2535,7 +2910,7 @@
       <c r="D14" s="145" t="n">
         <v>0.35</v>
       </c>
-      <c r="E14" s="172" t="n">
+      <c r="E14" s="180" t="n">
         <v>1.4</v>
       </c>
       <c r="F14" s="53" t="n">
@@ -2662,7 +3037,7 @@
           <t>Landed cost today, 4 SKUs (Vegetable, Spicy, Beef, Chicken), €/pack</t>
         </is>
       </c>
-      <c r="B23" s="173" t="n">
+      <c r="B23" s="181" t="n">
         <v>0.882380333698031</v>
       </c>
     </row>
@@ -2672,7 +3047,7 @@
           <t>Landed cost today, 2 SKUs (Gouda, Carbonara), €/pack</t>
         </is>
       </c>
-      <c r="B24" s="173" t="n">
+      <c r="B24" s="181" t="n">
         <v>1.018131154266958</v>
       </c>
     </row>

</xml_diff>

<commit_message>
SIAS model: hide batch-cost input rows
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_SIAS_EN.xlsx
+++ b/RAMEN_FINMODEL_SIAS_EN.xlsx
@@ -2341,7 +2341,7 @@
         <v>51.2</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" hidden="1" s="71">
       <c r="B15" s="45" t="inlineStr">
         <is>
           <t>Import VAT</t>
@@ -2373,7 +2373,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" hidden="1" s="71">
       <c r="B16" s="145" t="n">
         <v>0.2</v>
       </c>
@@ -2393,7 +2393,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" ht="20.4" customHeight="1" s="71">
+    <row r="17" hidden="1" ht="20.4" customHeight="1" s="71">
       <c r="B17" s="45" t="inlineStr">
         <is>
           <t>Freight share in customs value</t>
@@ -2410,7 +2410,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" hidden="1" s="71">
       <c r="B18" s="53" t="n">
         <v>0.7</v>
       </c>
@@ -2917,7 +2917,7 @@
         <v>51.2</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" hidden="1" s="71">
       <c r="B15" s="45" t="inlineStr">
         <is>
           <t>Import VAT</t>
@@ -2949,7 +2949,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" hidden="1" s="71">
       <c r="B16" s="145" t="n">
         <v>0.2</v>
       </c>
@@ -2969,7 +2969,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" ht="20.4" customHeight="1" s="71">
+    <row r="17" hidden="1" ht="20.4" customHeight="1" s="71">
       <c r="B17" s="45" t="inlineStr">
         <is>
           <t>Freight share in customs value</t>
@@ -2986,7 +2986,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" hidden="1" s="71">
       <c r="B18" s="53" t="n">
         <v>0.7</v>
       </c>

</xml_diff>

<commit_message>
SIAS model: remove batch-cost input rows (formulas use constants)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_SIAS_EN.xlsx
+++ b/RAMEN_FINMODEL_SIAS_EN.xlsx
@@ -1725,15 +1725,15 @@
         <v>27.648000000000003</v>
       </c>
       <c r="C8" s="178">
-        <f>('33 pallets'!E16+'33 pallets'!F16+'33 pallets'!G16)/('33 pallets'!C18*'33 pallets'!D18)*'33 pallets'!F14</f>
+        <f>(3700+288+42)/52800*'33 pallets'!F14</f>
         <v>3.907878787878788</v>
       </c>
       <c r="D8" s="178">
-        <f>('33 pallets'!B19+'33 pallets'!E16*'33 pallets'!B18/('33 pallets'!C18*'33 pallets'!D18))*(1+'33 pallets'!D16)*'33 pallets'!B16*'33 pallets'!F14</f>
+        <f>('33 pallets'!B19+3700*0.7/52800)*(1+0)*0.2*'33 pallets'!F14</f>
         <v>6.031903030303031</v>
       </c>
       <c r="E8" s="178">
-        <f>(B8+C8+D8+('33 pallets'!B19+'33 pallets'!E16*'33 pallets'!B18/('33 pallets'!C18*'33 pallets'!D18))*'33 pallets'!D16*'33 pallets'!F14)*'33 pallets'!C16</f>
+        <f>(B8+C8+D8+('33 pallets'!B19+3700*0.7/52800)*0*'33 pallets'!F14)*0.025</f>
         <v>0.9396945454545457</v>
       </c>
       <c r="F8" s="179">
@@ -1874,15 +1874,15 @@
         <v>16.384</v>
       </c>
       <c r="C14" s="178">
-        <f>('6 pallets'!E16+'6 pallets'!F16+'6 pallets'!G16)/('6 pallets'!C18*'6 pallets'!D18)*'6 pallets'!F14</f>
+        <f>(2600+288+42)/9600*'6 pallets'!F14</f>
         <v>15.626666666666669</v>
       </c>
       <c r="D14" s="178">
-        <f>('6 pallets'!B20+'6 pallets'!E16*'6 pallets'!B18/('6 pallets'!C18*'6 pallets'!D18))*(1+'6 pallets'!D16)*'6 pallets'!B16*'6 pallets'!F14</f>
+        <f>('6 pallets'!B20+2600*0.7/9600)*(1+0)*0.2*'6 pallets'!F14</f>
         <v>5.218133333333333</v>
       </c>
       <c r="E14" s="178">
-        <f>(B14+C14+D14+('6 pallets'!B20+'6 pallets'!E16*'6 pallets'!B18/('6 pallets'!C18*'6 pallets'!D18))*'6 pallets'!D16*'6 pallets'!F14)*'6 pallets'!C16</f>
+        <f>(B14+C14+D14+('6 pallets'!B20+2600*0.7/9600)*0*'6 pallets'!F14)*0.025</f>
         <v>0.93072</v>
       </c>
       <c r="F14" s="179">
@@ -1922,7 +1922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="38" customWidth="1" style="71" min="1" max="1"/>
@@ -2341,86 +2341,10 @@
         <v>51.2</v>
       </c>
     </row>
-    <row r="15" hidden="1" s="71">
-      <c r="B15" s="45" t="inlineStr">
-        <is>
-          <t>Import VAT</t>
-        </is>
-      </c>
-      <c r="C15" s="45" t="inlineStr">
-        <is>
-          <t>Financing</t>
-        </is>
-      </c>
-      <c r="D15" s="45" t="inlineStr">
-        <is>
-          <t>Customs duty</t>
-        </is>
-      </c>
-      <c r="E15" s="45" t="inlineStr">
-        <is>
-          <t>Batch freight, €</t>
-        </is>
-      </c>
-      <c r="F15" s="45" t="inlineStr">
-        <is>
-          <t>Broker, €</t>
-        </is>
-      </c>
-      <c r="G15" s="45" t="inlineStr">
-        <is>
-          <t>Other, €</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" hidden="1" s="71">
-      <c r="B16" s="145" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C16" s="145" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="D16" s="145" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="52" t="n">
-        <v>2600</v>
-      </c>
-      <c r="F16" s="52" t="n">
-        <v>288</v>
-      </c>
-      <c r="G16" s="52" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="17" hidden="1" ht="20.4" customHeight="1" s="71">
-      <c r="B17" s="45" t="inlineStr">
-        <is>
-          <t>Freight share in customs value</t>
-        </is>
-      </c>
-      <c r="C17" s="45" t="inlineStr">
-        <is>
-          <t>Pallets in batch</t>
-        </is>
-      </c>
-      <c r="D17" s="45" t="inlineStr">
-        <is>
-          <t>Packs per pallet</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" hidden="1" s="71">
-      <c r="B18" s="53" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="C18" s="52" t="n">
-        <v>6</v>
-      </c>
-      <c r="D18" s="52" t="n">
-        <v>1600</v>
-      </c>
-    </row>
+    <row r="15" ht="3" customHeight="1" s="71"/>
+    <row r="16" ht="3" customHeight="1" s="71"/>
+    <row r="17" ht="3" customHeight="1" s="71"/>
+    <row r="18" ht="3" customHeight="1" s="71"/>
     <row r="19"/>
     <row r="20">
       <c r="A20" s="54" t="inlineStr">
@@ -2429,7 +2353,7 @@
         </is>
       </c>
       <c r="B20" s="147">
-        <f>ROUNDDOWN(((B14/E14*(1-D14-C14))/F14/(1+C16)-(E16+F16+G16+E16*B18*(D16+B16*(1+D16)))/(C18*D18))/((1+D16)*(1+B16)),2)</f>
+        <f>ROUNDDOWN(((B14/E14*(1-D14-C14))/F14/(1+0.025)-(2600+288+42+2600*0.7*(0+0.2*(1+0)))/9600)/((1+0)*(1+0.2)),2)</f>
         <v>0.32</v>
       </c>
     </row>
@@ -2440,7 +2364,7 @@
         </is>
       </c>
       <c r="B21" s="148">
-        <f>((B14/E14*(1-D14-C14))/F14/(1+C16)-(E16+F16+G16+E16*B18*(D16+B16*(1+D16)))/(C18*D18))/((1+D16)*(1+B16))</f>
+        <f>((B14/E14*(1-D14-C14))/F14/(1+0.025)-(2600+288+42+2600*0.7*(0+0.2*(1+0)))/9600)/((1+0)*(1+0.2))</f>
         <v>0.3265407229965157</v>
       </c>
     </row>
@@ -2451,7 +2375,7 @@
         </is>
       </c>
       <c r="B22" s="57">
-        <f>(B20*F14+(E16+F16+G16)/(C18*D18)*F14+(B20+E16*B18/(C18*D18))*D16*F14+(B20+E16*B18/(C18*D18))*(1+D16)*B16*F14)*(1+C16)</f>
+        <f>(B20*F14+(2600+288+42)/9600*F14+(B20+2600*0.7/9600)*0*F14+(B20+2600*0.7/9600)*(1+0)*0.2*F14)*(1+0.025)</f>
         <v>38.15951999999999</v>
       </c>
     </row>
@@ -2500,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="38" customWidth="1" style="71" min="1" max="1"/>
@@ -2917,86 +2841,10 @@
         <v>51.2</v>
       </c>
     </row>
-    <row r="15" hidden="1" s="71">
-      <c r="B15" s="45" t="inlineStr">
-        <is>
-          <t>Import VAT</t>
-        </is>
-      </c>
-      <c r="C15" s="45" t="inlineStr">
-        <is>
-          <t>Financing</t>
-        </is>
-      </c>
-      <c r="D15" s="45" t="inlineStr">
-        <is>
-          <t>Customs duty</t>
-        </is>
-      </c>
-      <c r="E15" s="45" t="inlineStr">
-        <is>
-          <t>Batch freight, €</t>
-        </is>
-      </c>
-      <c r="F15" s="45" t="inlineStr">
-        <is>
-          <t>Broker, €</t>
-        </is>
-      </c>
-      <c r="G15" s="45" t="inlineStr">
-        <is>
-          <t>Other, €</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" hidden="1" s="71">
-      <c r="B16" s="145" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C16" s="145" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="D16" s="145" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="52" t="n">
-        <v>3700</v>
-      </c>
-      <c r="F16" s="52" t="n">
-        <v>288</v>
-      </c>
-      <c r="G16" s="52" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="17" hidden="1" ht="20.4" customHeight="1" s="71">
-      <c r="B17" s="45" t="inlineStr">
-        <is>
-          <t>Freight share in customs value</t>
-        </is>
-      </c>
-      <c r="C17" s="45" t="inlineStr">
-        <is>
-          <t>Pallets in batch</t>
-        </is>
-      </c>
-      <c r="D17" s="45" t="inlineStr">
-        <is>
-          <t>Packs per pallet</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" hidden="1" s="71">
-      <c r="B18" s="53" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="C18" s="52" t="n">
-        <v>33</v>
-      </c>
-      <c r="D18" s="52" t="n">
-        <v>1600</v>
-      </c>
-    </row>
+    <row r="15" ht="3" customHeight="1" s="71"/>
+    <row r="16" ht="3" customHeight="1" s="71"/>
+    <row r="17" ht="3" customHeight="1" s="71"/>
+    <row r="18" ht="3" customHeight="1" s="71"/>
     <row r="19">
       <c r="A19" s="54" t="inlineStr">
         <is>
@@ -3004,7 +2852,7 @@
         </is>
       </c>
       <c r="B19" s="147">
-        <f>ROUNDDOWN(((B14/E14*(1-D14-C14))/F14/(1+C16)-(E16+F16+G16+E16*B18*(D16+B16*(1+D16)))/(C18*D18))/((1+D16)*(1+B16)),2)</f>
+        <f>ROUNDDOWN(((B14/E14*(1-D14-C14))/F14/(1+0.025)-(3700+288+42+3700*0.7*(0+0.2*(1+0)))/52800)/((1+0)*(1+0.2)),2)</f>
         <v>0.54</v>
       </c>
     </row>
@@ -3015,7 +2863,7 @@
         </is>
       </c>
       <c r="B20" s="148">
-        <f>((B14/E14*(1-D14-C14))/F14/(1+C16)-(E16+F16+G16+E16*B18*(D16+B16*(1+D16)))/(C18*D18))/((1+D16)*(1+B16))</f>
+        <f>((B14/E14*(1-D14-C14))/F14/(1+0.025)-(3700+288+42+3700*0.7*(0+0.2*(1+0)))/52800)/((1+0)*(1+0.2))</f>
         <v>0.5406979199662126</v>
       </c>
     </row>
@@ -3026,7 +2874,7 @@
         </is>
       </c>
       <c r="B21" s="57">
-        <f>(B19*F14+(E16+F16+G16)/(C18*D18)*F14+(B19+E16*B18/(C18*D18))*D16*F14+(B19+E16*B18/(C18*D18))*(1+D16)*B16*F14)*(1+C16)</f>
+        <f>(B19*F14+(3700+288+42)/52800*F14+(B19+3700*0.7/52800)*0*F14+(B19+3700*0.7/52800)*(1+0)*0.2*F14)*(1+0.025)</f>
         <v>38.52747636363637</v>
       </c>
     </row>

</xml_diff>